<commit_message>
implement download excel file
</commit_message>
<xml_diff>
--- a/application/static/excel/import-file.xlsx
+++ b/application/static/excel/import-file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liengphuto/workspace/hanatools/shield-check/application/static/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A8E6CD-D1E9-2341-BCEC-6167EF816F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E53711E-2178-EB44-BFDC-64BC1211D8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2860" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{C396972B-5BA1-D040-82BA-FE76C7FAEC89}"/>
+    <workbookView xWindow="2660" yWindow="2860" windowWidth="28040" windowHeight="17440" xr2:uid="{C396972B-5BA1-D040-82BA-FE76C7FAEC89}"/>
   </bookViews>
   <sheets>
     <sheet name="member" sheetId="1" r:id="rId1"/>

</xml_diff>